<commit_message>
working on charts formula's
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/3_Logical_Functions.xlsx
+++ b/2_Formulas_Functions/3_Logical_Functions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DataAnalytics\Excel_Data_Analytics\2_Formulas_Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32D91ADC-AFF3-4CDB-B211-05C0A7A062A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE421459-834F-4A32-875B-9D83AE139A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8CC555B5-3E06-43B6-9E5B-C0A1D3498DA4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{8CC555B5-3E06-43B6-9E5B-C0A1D3498DA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_1" sheetId="7" r:id="rId1"/>
@@ -25,7 +25,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Final_2!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1325,15 +1324,15 @@
     <col min="3" max="3" width="18.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.21875" style="1" customWidth="1"/>
     <col min="5" max="5" width="11.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" style="1" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="8" max="9" width="11.109375" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="17.21875" style="1" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="14.21875" style="1" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="1" customWidth="1"/>
+    <col min="8" max="9" width="11.109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.21875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.21875" style="1" customWidth="1"/>
     <col min="13" max="13" width="9.109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="10.44140625" style="1" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="14.109375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="10.44140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="14.109375" style="1" customWidth="1"/>
     <col min="16" max="16" width="9.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="9.109375" style="1"/>
     <col min="18" max="18" width="14.109375" style="1" bestFit="1" customWidth="1"/>

</xml_diff>